<commit_message>
Clean up the markers
</commit_message>
<xml_diff>
--- a/locations.xlsx
+++ b/locations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\retro\repos\quest-rfi-new-sites\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EFACA6D-2FF2-4B96-965C-F3958A1071DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4EE63BC-6B9E-4004-8638-2BD05ACADA4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5460" yWindow="3735" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3210" yWindow="2970" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sample Sites RFI" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1266" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1267" uniqueCount="29">
   <si>
     <t>ID RFI</t>
   </si>
@@ -124,6 +124,9 @@
   </si>
   <si>
     <t>required_height</t>
+  </si>
+  <si>
+    <t>s</t>
   </si>
 </sst>
 </file>
@@ -503,7 +506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED183A52-6DC1-47D7-A90E-AA6976A9EB2E}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E107"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
@@ -530,8 +533,8 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="4">
-        <v>8.8932739999999999</v>
+      <c r="A2" s="4" t="s">
+        <v>28</v>
       </c>
       <c r="B2" s="4">
         <v>-79.620080999999999</v>
@@ -565,16 +568,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
-        <v>9.0798469999999991</v>
+        <v>7.984642</v>
       </c>
       <c r="B4" s="4">
-        <v>-79.42859</v>
+        <v>-80.432357999999994</v>
       </c>
       <c r="C4" s="3">
         <v>500</v>
       </c>
       <c r="D4" s="3">
-        <v>372</v>
+        <v>89</v>
       </c>
       <c r="E4" s="3">
         <v>15</v>
@@ -582,36 +585,1753 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
-        <v>9.3435000000000006</v>
+        <v>8.3496830000000006</v>
       </c>
       <c r="B5" s="4">
-        <v>-82.250470000000007</v>
+        <v>-80.171053999999998</v>
       </c>
       <c r="C5" s="3">
         <v>500</v>
       </c>
       <c r="D5" s="3">
-        <v>373</v>
+        <v>96</v>
       </c>
       <c r="E5" s="3">
-        <v>25</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
+        <v>9.0219719999999999</v>
+      </c>
+      <c r="B6" s="4">
+        <v>-79.477215999999999</v>
+      </c>
+      <c r="C6" s="3">
+        <v>250</v>
+      </c>
+      <c r="D6" s="3">
+        <v>102</v>
+      </c>
+      <c r="E6" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>8.3307099999999998</v>
+      </c>
+      <c r="B7" s="4">
+        <v>-80.517799999999994</v>
+      </c>
+      <c r="C7" s="3">
+        <v>500</v>
+      </c>
+      <c r="D7" s="3">
+        <v>108</v>
+      </c>
+      <c r="E7" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>8.9763369999999991</v>
+      </c>
+      <c r="B8" s="4">
+        <v>-79.507999999999996</v>
+      </c>
+      <c r="C8" s="3">
+        <v>250</v>
+      </c>
+      <c r="D8" s="3">
+        <v>140</v>
+      </c>
+      <c r="E8" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="4">
+        <v>8.9710300000000007</v>
+      </c>
+      <c r="B9" s="4">
+        <v>-79.534639999999996</v>
+      </c>
+      <c r="C9" s="3">
+        <v>250</v>
+      </c>
+      <c r="D9" s="3">
+        <v>179</v>
+      </c>
+      <c r="E9" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>9.0269069999999996</v>
+      </c>
+      <c r="B10" s="4">
+        <v>-79.480800000000002</v>
+      </c>
+      <c r="C10" s="3">
+        <v>500</v>
+      </c>
+      <c r="D10" s="3">
+        <v>180</v>
+      </c>
+      <c r="E10" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>8.9954400000000003</v>
+      </c>
+      <c r="B11" s="4">
+        <v>-79.531559999999999</v>
+      </c>
+      <c r="C11" s="3">
+        <v>250</v>
+      </c>
+      <c r="D11" s="3">
+        <v>183</v>
+      </c>
+      <c r="E11" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
+        <v>8.9566199999999991</v>
+      </c>
+      <c r="B12" s="4">
+        <v>-79.541550000000001</v>
+      </c>
+      <c r="C12" s="3">
+        <v>250</v>
+      </c>
+      <c r="D12" s="3">
+        <v>185</v>
+      </c>
+      <c r="E12" s="3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="4">
+        <v>9.0062479999999994</v>
+      </c>
+      <c r="B13" s="4">
+        <v>-79.537760000000006</v>
+      </c>
+      <c r="C13" s="3">
+        <v>250</v>
+      </c>
+      <c r="D13" s="3">
+        <v>186</v>
+      </c>
+      <c r="E13" s="3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>9.1670449999999999</v>
+      </c>
+      <c r="B14" s="4">
+        <v>-79.536792000000005</v>
+      </c>
+      <c r="C14" s="3">
+        <v>500</v>
+      </c>
+      <c r="D14" s="3">
+        <v>187</v>
+      </c>
+      <c r="E14" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
+        <v>9.0462699999999998</v>
+      </c>
+      <c r="B15" s="4">
+        <v>-79.446089999999998</v>
+      </c>
+      <c r="C15" s="3">
+        <v>250</v>
+      </c>
+      <c r="D15" s="3">
+        <v>188</v>
+      </c>
+      <c r="E15" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="4">
+        <v>8.5422980000000006</v>
+      </c>
+      <c r="B16" s="4">
+        <v>-79.914688999999996</v>
+      </c>
+      <c r="C16" s="3">
+        <v>250</v>
+      </c>
+      <c r="D16" s="3">
+        <v>189</v>
+      </c>
+      <c r="E16" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="4">
+        <v>9.0496409999999994</v>
+      </c>
+      <c r="B17" s="4">
+        <v>-79.634500000000003</v>
+      </c>
+      <c r="C17" s="3">
+        <v>750</v>
+      </c>
+      <c r="D17" s="3">
+        <v>191</v>
+      </c>
+      <c r="E17" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="4">
+        <v>8.9668679999999998</v>
+      </c>
+      <c r="B18" s="4">
+        <v>-79.539919999999995</v>
+      </c>
+      <c r="C18" s="3">
+        <v>250</v>
+      </c>
+      <c r="D18" s="3">
+        <v>194</v>
+      </c>
+      <c r="E18" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="4">
+        <v>8.4292400000000001</v>
+      </c>
+      <c r="B19" s="4">
+        <v>-82.429469999999995</v>
+      </c>
+      <c r="C19" s="3">
+        <v>250</v>
+      </c>
+      <c r="D19" s="3">
+        <v>196</v>
+      </c>
+      <c r="E19" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="4">
+        <v>9.0591249999999999</v>
+      </c>
+      <c r="B20" s="4">
+        <v>-79.431079999999994</v>
+      </c>
+      <c r="C20" s="3">
+        <v>250</v>
+      </c>
+      <c r="D20" s="3">
+        <v>197</v>
+      </c>
+      <c r="E20" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="4">
+        <v>8.9819359999999993</v>
+      </c>
+      <c r="B21" s="4">
+        <v>-79.518709999999999</v>
+      </c>
+      <c r="C21" s="3">
+        <v>250</v>
+      </c>
+      <c r="D21" s="3">
+        <v>201</v>
+      </c>
+      <c r="E21" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="4">
+        <v>9.0129380000000001</v>
+      </c>
+      <c r="B22" s="4">
+        <v>-79.492230000000006</v>
+      </c>
+      <c r="C22" s="3">
+        <v>500</v>
+      </c>
+      <c r="D22" s="3">
+        <v>211</v>
+      </c>
+      <c r="E22" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="4">
+        <v>9.0307729999999999</v>
+      </c>
+      <c r="B23" s="4">
+        <v>-79.522509999999997</v>
+      </c>
+      <c r="C23" s="3">
+        <v>250</v>
+      </c>
+      <c r="D23" s="3">
+        <v>214</v>
+      </c>
+      <c r="E23" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="4">
+        <v>9.0012100000000004</v>
+      </c>
+      <c r="B24" s="4">
+        <v>-79.583629999999999</v>
+      </c>
+      <c r="C24" s="3">
+        <v>500</v>
+      </c>
+      <c r="D24" s="3">
+        <v>233</v>
+      </c>
+      <c r="E24" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="4">
+        <v>8.9759910000000005</v>
+      </c>
+      <c r="B25" s="4">
+        <v>-79.521889999999999</v>
+      </c>
+      <c r="C25" s="3">
+        <v>250</v>
+      </c>
+      <c r="D25" s="3">
+        <v>250</v>
+      </c>
+      <c r="E25" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="4">
+        <v>9.0172220000000003</v>
+      </c>
+      <c r="B26" s="4">
+        <v>-79.502028999999993</v>
+      </c>
+      <c r="C26" s="3">
+        <v>250</v>
+      </c>
+      <c r="D26" s="3">
+        <v>255</v>
+      </c>
+      <c r="E26" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="4">
+        <v>8.9823500000000003</v>
+      </c>
+      <c r="B27" s="4">
+        <v>-79.511179999999996</v>
+      </c>
+      <c r="C27" s="3">
+        <v>250</v>
+      </c>
+      <c r="D27" s="3">
+        <v>262</v>
+      </c>
+      <c r="E27" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="4">
+        <v>9.0239189999999994</v>
+      </c>
+      <c r="B28" s="4">
+        <v>-79.487271000000007</v>
+      </c>
+      <c r="C28" s="3">
+        <v>250</v>
+      </c>
+      <c r="D28" s="3">
+        <v>263</v>
+      </c>
+      <c r="E28" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="4">
+        <v>8.9625079999999997</v>
+      </c>
+      <c r="B29" s="4">
+        <v>-79.543940000000006</v>
+      </c>
+      <c r="C29" s="3">
+        <v>250</v>
+      </c>
+      <c r="D29" s="3">
+        <v>266</v>
+      </c>
+      <c r="E29" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="4">
+        <v>8.9762199999999996</v>
+      </c>
+      <c r="B30" s="4">
+        <v>-79.525729999999996</v>
+      </c>
+      <c r="C30" s="3">
+        <v>250</v>
+      </c>
+      <c r="D30" s="3">
+        <v>279</v>
+      </c>
+      <c r="E30" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="4">
+        <v>9.0149720000000002</v>
+      </c>
+      <c r="B31" s="4">
+        <v>-79.517669999999995</v>
+      </c>
+      <c r="C31" s="3">
+        <v>250</v>
+      </c>
+      <c r="D31" s="3">
+        <v>282</v>
+      </c>
+      <c r="E31" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="4">
+        <v>9.0194200000000002</v>
+      </c>
+      <c r="B32" s="4">
+        <v>-79.533680000000004</v>
+      </c>
+      <c r="C32" s="3">
+        <v>250</v>
+      </c>
+      <c r="D32" s="3">
+        <v>285</v>
+      </c>
+      <c r="E32" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="4">
+        <v>8.9624199999999998</v>
+      </c>
+      <c r="B33" s="4">
+        <v>-79.537310000000005</v>
+      </c>
+      <c r="C33" s="3">
+        <v>250</v>
+      </c>
+      <c r="D33" s="3">
+        <v>292</v>
+      </c>
+      <c r="E33" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="4">
+        <v>8.9716699999999996</v>
+      </c>
+      <c r="B34" s="4">
+        <v>-79.531490000000005</v>
+      </c>
+      <c r="C34" s="3">
+        <v>250</v>
+      </c>
+      <c r="D34" s="3">
+        <v>295</v>
+      </c>
+      <c r="E34" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="4">
+        <v>8.9877300000000009</v>
+      </c>
+      <c r="B35" s="4">
+        <v>-79.503270000000001</v>
+      </c>
+      <c r="C35" s="3">
+        <v>250</v>
+      </c>
+      <c r="D35" s="3">
+        <v>300</v>
+      </c>
+      <c r="E35" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="4">
+        <v>9.0694529999999993</v>
+      </c>
+      <c r="B36" s="4">
+        <v>-79.463308999999995</v>
+      </c>
+      <c r="C36" s="3">
+        <v>250</v>
+      </c>
+      <c r="D36" s="3">
+        <v>315</v>
+      </c>
+      <c r="E36" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="4">
+        <v>8.9056119999999996</v>
+      </c>
+      <c r="B37" s="4">
+        <v>-79.782380000000003</v>
+      </c>
+      <c r="C37" s="3">
+        <v>500</v>
+      </c>
+      <c r="D37" s="3">
+        <v>320</v>
+      </c>
+      <c r="E37" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="4">
+        <v>9.0632129999999993</v>
+      </c>
+      <c r="B38" s="4">
+        <v>-79.433610000000002</v>
+      </c>
+      <c r="C38" s="3">
+        <v>500</v>
+      </c>
+      <c r="D38" s="3">
+        <v>321</v>
+      </c>
+      <c r="E38" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="4">
+        <v>9.1156559999999995</v>
+      </c>
+      <c r="B39" s="4">
+        <v>-79.354894999999999</v>
+      </c>
+      <c r="C39" s="3">
+        <v>500</v>
+      </c>
+      <c r="D39" s="3">
+        <v>322</v>
+      </c>
+      <c r="E39" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="4">
+        <v>9.1164299999999994</v>
+      </c>
+      <c r="B40" s="4">
+        <v>-79.575450000000004</v>
+      </c>
+      <c r="C40" s="3">
+        <v>500</v>
+      </c>
+      <c r="D40" s="3">
+        <v>323</v>
+      </c>
+      <c r="E40" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="4">
+        <v>8.9986099999999993</v>
+      </c>
+      <c r="B41" s="4">
+        <v>-79.533829999999995</v>
+      </c>
+      <c r="C41" s="3">
+        <v>250</v>
+      </c>
+      <c r="D41" s="3">
+        <v>324</v>
+      </c>
+      <c r="E41" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="4">
+        <v>8.999174</v>
+      </c>
+      <c r="B42" s="4">
+        <v>-79.513914999999997</v>
+      </c>
+      <c r="C42" s="3">
+        <v>250</v>
+      </c>
+      <c r="D42" s="3">
+        <v>325</v>
+      </c>
+      <c r="E42" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="4">
+        <v>8.9675200000000004</v>
+      </c>
+      <c r="B43" s="4">
+        <v>-79.541309999999996</v>
+      </c>
+      <c r="C43" s="3">
+        <v>250</v>
+      </c>
+      <c r="D43" s="3">
+        <v>326</v>
+      </c>
+      <c r="E43" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="4">
+        <v>8.9537999999999993</v>
+      </c>
+      <c r="B44" s="4">
+        <v>-79.581850000000003</v>
+      </c>
+      <c r="C44" s="3">
+        <v>250</v>
+      </c>
+      <c r="D44" s="3">
+        <v>327</v>
+      </c>
+      <c r="E44" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="4">
+        <v>7.7375559999999997</v>
+      </c>
+      <c r="B45" s="4">
+        <v>-80.247470000000007</v>
+      </c>
+      <c r="C45" s="3">
+        <v>500</v>
+      </c>
+      <c r="D45" s="3">
+        <v>328</v>
+      </c>
+      <c r="E45" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="4">
+        <v>8.0816569999999999</v>
+      </c>
+      <c r="B46" s="4">
+        <v>-80.915756999999999</v>
+      </c>
+      <c r="C46" s="3">
+        <v>750</v>
+      </c>
+      <c r="D46" s="3">
+        <v>329</v>
+      </c>
+      <c r="E46" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="4">
+        <v>8.1946049999999993</v>
+      </c>
+      <c r="B47" s="4">
+        <v>-82.876777000000004</v>
+      </c>
+      <c r="C47" s="3">
+        <v>1500</v>
+      </c>
+      <c r="D47" s="3">
+        <v>330</v>
+      </c>
+      <c r="E47" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="4">
+        <v>8.5527180000000005</v>
+      </c>
+      <c r="B48" s="4">
+        <v>-82.626052999999999</v>
+      </c>
+      <c r="C48" s="3">
+        <v>750</v>
+      </c>
+      <c r="D48" s="3">
+        <v>331</v>
+      </c>
+      <c r="E48" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="4">
+        <v>9.1331220000000002</v>
+      </c>
+      <c r="B49" s="4">
+        <v>-79.225949999999997</v>
+      </c>
+      <c r="C49" s="3">
+        <v>500</v>
+      </c>
+      <c r="D49" s="3">
+        <v>332</v>
+      </c>
+      <c r="E49" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="4">
+        <v>9.0940449999999995</v>
+      </c>
+      <c r="B50" s="4">
+        <v>-79.508930000000007</v>
+      </c>
+      <c r="C50" s="3">
+        <v>500</v>
+      </c>
+      <c r="D50" s="3">
+        <v>333</v>
+      </c>
+      <c r="E50" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="4">
+        <v>9.0839040000000004</v>
+      </c>
+      <c r="B51" s="4">
+        <v>-79.501440000000002</v>
+      </c>
+      <c r="C51" s="3">
+        <v>500</v>
+      </c>
+      <c r="D51" s="3">
+        <v>334</v>
+      </c>
+      <c r="E51" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="4">
+        <v>9.3511000000000006</v>
+      </c>
+      <c r="B52" s="4">
+        <v>-79.815579999999997</v>
+      </c>
+      <c r="C52" s="3">
+        <v>500</v>
+      </c>
+      <c r="D52" s="3">
+        <v>335</v>
+      </c>
+      <c r="E52" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="4">
+        <v>9.0371590000000008</v>
+      </c>
+      <c r="B53" s="4">
+        <v>-79.419134</v>
+      </c>
+      <c r="C53" s="3">
+        <v>500</v>
+      </c>
+      <c r="D53" s="3">
+        <v>336</v>
+      </c>
+      <c r="E53" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="4">
+        <v>9.0785</v>
+      </c>
+      <c r="B54" s="4">
+        <v>-79.460499999999996</v>
+      </c>
+      <c r="C54" s="3">
+        <v>500</v>
+      </c>
+      <c r="D54" s="3">
+        <v>337</v>
+      </c>
+      <c r="E54" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="4">
+        <v>7.96739</v>
+      </c>
+      <c r="B55" s="4">
+        <v>-80.469268</v>
+      </c>
+      <c r="C55" s="3">
+        <v>750</v>
+      </c>
+      <c r="D55" s="3">
+        <v>338</v>
+      </c>
+      <c r="E55" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="4">
+        <v>9.1118799999999993</v>
+      </c>
+      <c r="B56" s="4">
+        <v>-79.328580000000002</v>
+      </c>
+      <c r="C56" s="3">
+        <v>500</v>
+      </c>
+      <c r="D56" s="3">
+        <v>339</v>
+      </c>
+      <c r="E56" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="4">
+        <v>9.0294919999999994</v>
+      </c>
+      <c r="B57" s="4">
+        <v>-79.455659999999995</v>
+      </c>
+      <c r="C57" s="3">
+        <v>500</v>
+      </c>
+      <c r="D57" s="3">
+        <v>340</v>
+      </c>
+      <c r="E57" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" s="4">
+        <v>9.0514609999999998</v>
+      </c>
+      <c r="B58" s="4">
+        <v>-79.444310000000002</v>
+      </c>
+      <c r="C58" s="3">
+        <v>500</v>
+      </c>
+      <c r="D58" s="3">
+        <v>341</v>
+      </c>
+      <c r="E58" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="4">
+        <v>8.8055830000000004</v>
+      </c>
+      <c r="B59" s="4">
+        <v>-79.895359999999997</v>
+      </c>
+      <c r="C59" s="3">
+        <v>750</v>
+      </c>
+      <c r="D59" s="3">
+        <v>342</v>
+      </c>
+      <c r="E59" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="4">
+        <v>8.7126889999999992</v>
+      </c>
+      <c r="B60" s="4">
+        <v>-79.880868000000007</v>
+      </c>
+      <c r="C60" s="3">
+        <v>750</v>
+      </c>
+      <c r="D60" s="3">
+        <v>343</v>
+      </c>
+      <c r="E60" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="4">
+        <v>9.043253</v>
+      </c>
+      <c r="B61" s="4">
+        <v>-79.443264999999997</v>
+      </c>
+      <c r="C61" s="3">
+        <v>250</v>
+      </c>
+      <c r="D61" s="3">
+        <v>344</v>
+      </c>
+      <c r="E61" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="4">
+        <v>9.1109449999999992</v>
+      </c>
+      <c r="B62" s="4">
+        <v>-79.336330000000004</v>
+      </c>
+      <c r="C62" s="3">
+        <v>250</v>
+      </c>
+      <c r="D62" s="3">
+        <v>345</v>
+      </c>
+      <c r="E62" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="4">
+        <v>8.078462</v>
+      </c>
+      <c r="B63" s="4">
+        <v>-80.936321000000007</v>
+      </c>
+      <c r="C63" s="3">
+        <v>500</v>
+      </c>
+      <c r="D63" s="3">
+        <v>346</v>
+      </c>
+      <c r="E63" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="4">
+        <v>8.9150749999999999</v>
+      </c>
+      <c r="B64" s="4">
+        <v>-79.530899000000005</v>
+      </c>
+      <c r="C64" s="3">
+        <v>500</v>
+      </c>
+      <c r="D64" s="3">
+        <v>347</v>
+      </c>
+      <c r="E64" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="4">
+        <v>9.0583860000000005</v>
+      </c>
+      <c r="B65" s="4">
+        <v>-79.506795999999994</v>
+      </c>
+      <c r="C65" s="3">
+        <v>500</v>
+      </c>
+      <c r="D65" s="3">
+        <v>348</v>
+      </c>
+      <c r="E65" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="4">
+        <v>8.9500770000000003</v>
+      </c>
+      <c r="B66" s="4">
+        <v>-79.550210000000007</v>
+      </c>
+      <c r="C66" s="3">
+        <v>250</v>
+      </c>
+      <c r="D66" s="3">
+        <v>349</v>
+      </c>
+      <c r="E66" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="4">
+        <v>9.0846789999999995</v>
+      </c>
+      <c r="B67" s="4">
+        <v>-79.397401000000002</v>
+      </c>
+      <c r="C67" s="3">
+        <v>500</v>
+      </c>
+      <c r="D67" s="3">
+        <v>350</v>
+      </c>
+      <c r="E67" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="4">
+        <v>9.0678409999999996</v>
+      </c>
+      <c r="B68" s="4">
+        <v>-79.426505000000006</v>
+      </c>
+      <c r="C68" s="3">
+        <v>500</v>
+      </c>
+      <c r="D68" s="3">
+        <v>351</v>
+      </c>
+      <c r="E68" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="4">
+        <v>8.877167</v>
+      </c>
+      <c r="B69" s="4">
+        <v>-79.763666999999998</v>
+      </c>
+      <c r="C69" s="3">
+        <v>500</v>
+      </c>
+      <c r="D69" s="3">
+        <v>352</v>
+      </c>
+      <c r="E69" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="4">
+        <v>9.0303109999999993</v>
+      </c>
+      <c r="B70" s="4">
+        <v>-79.490560000000002</v>
+      </c>
+      <c r="C70" s="3">
+        <v>250</v>
+      </c>
+      <c r="D70" s="3">
+        <v>353</v>
+      </c>
+      <c r="E70" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="4">
+        <v>9.0453670000000006</v>
+      </c>
+      <c r="B71" s="4">
+        <v>-79.471566999999993</v>
+      </c>
+      <c r="C71" s="3">
+        <v>250</v>
+      </c>
+      <c r="D71" s="3">
+        <v>354</v>
+      </c>
+      <c r="E71" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="4">
+        <v>8.5294899999999991</v>
+      </c>
+      <c r="B72" s="4">
+        <v>-79.915819999999997</v>
+      </c>
+      <c r="C72" s="3">
+        <v>500</v>
+      </c>
+      <c r="D72" s="3">
+        <v>355</v>
+      </c>
+      <c r="E72" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="4">
+        <v>8.9023330000000005</v>
+      </c>
+      <c r="B73" s="4">
+        <v>-79.752691999999996</v>
+      </c>
+      <c r="C73" s="3">
+        <v>500</v>
+      </c>
+      <c r="D73" s="3">
+        <v>356</v>
+      </c>
+      <c r="E73" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="4">
+        <v>9.0919399999999992</v>
+      </c>
+      <c r="B74" s="4">
+        <v>-79.498239999999996</v>
+      </c>
+      <c r="C74" s="3">
+        <v>500</v>
+      </c>
+      <c r="D74" s="3">
+        <v>357</v>
+      </c>
+      <c r="E74" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="4">
+        <v>9.0726320000000005</v>
+      </c>
+      <c r="B75" s="4">
+        <v>-79.487560000000002</v>
+      </c>
+      <c r="C75" s="3">
+        <v>500</v>
+      </c>
+      <c r="D75" s="3">
+        <v>358</v>
+      </c>
+      <c r="E75" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="4">
+        <v>8.4323499999999996</v>
+      </c>
+      <c r="B76" s="4">
+        <v>-82.457279999999997</v>
+      </c>
+      <c r="C76" s="3">
+        <v>500</v>
+      </c>
+      <c r="D76" s="3">
+        <v>359</v>
+      </c>
+      <c r="E76" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="4">
+        <v>9.0495000000000001</v>
+      </c>
+      <c r="B77" s="4">
+        <v>-79.504549999999995</v>
+      </c>
+      <c r="C77" s="3">
+        <v>250</v>
+      </c>
+      <c r="D77" s="3">
+        <v>360</v>
+      </c>
+      <c r="E77" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="4">
+        <v>7.7545120000000001</v>
+      </c>
+      <c r="B78" s="4">
+        <v>-80.268681999999998</v>
+      </c>
+      <c r="C78" s="3">
+        <v>500</v>
+      </c>
+      <c r="D78" s="3">
+        <v>361</v>
+      </c>
+      <c r="E78" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="4">
+        <v>8.5556110000000007</v>
+      </c>
+      <c r="B79" s="4">
+        <v>-80.324640000000002</v>
+      </c>
+      <c r="C79" s="3">
+        <v>750</v>
+      </c>
+      <c r="D79" s="3">
+        <v>362</v>
+      </c>
+      <c r="E79" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="4">
+        <v>8.8296299999999999</v>
+      </c>
+      <c r="B80" s="4">
+        <v>-79.790599999999998</v>
+      </c>
+      <c r="C80" s="3">
+        <v>500</v>
+      </c>
+      <c r="D80" s="3">
+        <v>363</v>
+      </c>
+      <c r="E80" s="3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="4">
+        <v>8.2314989999999995</v>
+      </c>
+      <c r="B81" s="4">
+        <v>-80.538917999999995</v>
+      </c>
+      <c r="C81" s="3">
+        <v>500</v>
+      </c>
+      <c r="D81" s="3">
+        <v>364</v>
+      </c>
+      <c r="E81" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="4">
+        <v>9.0389090000000003</v>
+      </c>
+      <c r="B82" s="4">
+        <v>-79.507750000000001</v>
+      </c>
+      <c r="C82" s="3">
+        <v>250</v>
+      </c>
+      <c r="D82" s="3">
+        <v>365</v>
+      </c>
+      <c r="E82" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="4">
+        <v>8.2000879999999992</v>
+      </c>
+      <c r="B83" s="4">
+        <v>-80.627109000000004</v>
+      </c>
+      <c r="C83" s="3">
+        <v>750</v>
+      </c>
+      <c r="D83" s="3">
+        <v>366</v>
+      </c>
+      <c r="E83" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="4">
+        <v>8.3907100000000003</v>
+      </c>
+      <c r="B84" s="4">
+        <v>-80.260999999999996</v>
+      </c>
+      <c r="C84" s="3">
+        <v>500</v>
+      </c>
+      <c r="D84" s="3">
+        <v>367</v>
+      </c>
+      <c r="E84" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="4">
+        <v>9.0665790000000008</v>
+      </c>
+      <c r="B85" s="4">
+        <v>-79.414790999999994</v>
+      </c>
+      <c r="C85" s="3">
+        <v>500</v>
+      </c>
+      <c r="D85" s="3">
+        <v>368</v>
+      </c>
+      <c r="E85" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" s="4">
+        <v>8.9376840000000009</v>
+      </c>
+      <c r="B86" s="4">
+        <v>-79.729101</v>
+      </c>
+      <c r="C86" s="3">
+        <v>500</v>
+      </c>
+      <c r="D86" s="3">
+        <v>369</v>
+      </c>
+      <c r="E86" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" s="4">
+        <v>9.3583999999999996</v>
+      </c>
+      <c r="B87" s="4">
+        <v>-79.901388999999995</v>
+      </c>
+      <c r="C87" s="3">
+        <v>250</v>
+      </c>
+      <c r="D87" s="3">
+        <v>370</v>
+      </c>
+      <c r="E87" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" s="4">
+        <v>8.5177999999999994</v>
+      </c>
+      <c r="B88" s="4">
+        <v>-82.619399999999999</v>
+      </c>
+      <c r="C88" s="3">
+        <v>500</v>
+      </c>
+      <c r="D88" s="3">
+        <v>371</v>
+      </c>
+      <c r="E88" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" s="4">
+        <v>9.0798469999999991</v>
+      </c>
+      <c r="B89" s="4">
+        <v>-79.42859</v>
+      </c>
+      <c r="C89" s="3">
+        <v>500</v>
+      </c>
+      <c r="D89" s="3">
+        <v>372</v>
+      </c>
+      <c r="E89" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" s="4">
+        <v>9.3435000000000006</v>
+      </c>
+      <c r="B90" s="4">
+        <v>-82.250470000000007</v>
+      </c>
+      <c r="C90" s="3">
+        <v>500</v>
+      </c>
+      <c r="D90" s="3">
+        <v>373</v>
+      </c>
+      <c r="E90" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="4">
+        <v>9.0647079999999995</v>
+      </c>
+      <c r="B91" s="4">
+        <v>-79.442672000000002</v>
+      </c>
+      <c r="C91" s="3">
+        <v>500</v>
+      </c>
+      <c r="D91" s="3">
+        <v>374</v>
+      </c>
+      <c r="E91" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="4">
         <v>9.1020099999999999</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B92" s="4">
         <v>-79.542342000000005</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C92" s="3">
         <v>500</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D92" s="3">
         <v>453</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E92" s="3">
         <v>45</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" s="4">
+        <v>7.7553190000000001</v>
+      </c>
+      <c r="B93" s="4">
+        <v>-80.286081999999993</v>
+      </c>
+      <c r="C93" s="3">
+        <v>500</v>
+      </c>
+      <c r="D93" s="3">
+        <v>622</v>
+      </c>
+      <c r="E93" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" s="4">
+        <v>9.0978999999999992</v>
+      </c>
+      <c r="B94" s="4">
+        <v>-79.490200000000002</v>
+      </c>
+      <c r="C94" s="3">
+        <v>250</v>
+      </c>
+      <c r="D94" s="3">
+        <v>1233</v>
+      </c>
+      <c r="E94" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" s="4">
+        <v>8.9148300000000003</v>
+      </c>
+      <c r="B95" s="4">
+        <v>-79.522710000000004</v>
+      </c>
+      <c r="C95" s="3">
+        <v>250</v>
+      </c>
+      <c r="D95" s="3">
+        <v>1234</v>
+      </c>
+      <c r="E95" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" s="4">
+        <v>9.0707000000000004</v>
+      </c>
+      <c r="B96" s="4">
+        <v>-79.444450000000003</v>
+      </c>
+      <c r="C96" s="3">
+        <v>500</v>
+      </c>
+      <c r="D96" s="3">
+        <v>1235</v>
+      </c>
+      <c r="E96" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" s="4">
+        <v>8.5350699999999993</v>
+      </c>
+      <c r="B97" s="4">
+        <v>-82.838718</v>
+      </c>
+      <c r="C97" s="3">
+        <v>500</v>
+      </c>
+      <c r="D97" s="3">
+        <v>1236</v>
+      </c>
+      <c r="E97" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" s="4">
+        <v>7.9786999999999999</v>
+      </c>
+      <c r="B98" s="4">
+        <v>-80.456199999999995</v>
+      </c>
+      <c r="C98" s="3">
+        <v>500</v>
+      </c>
+      <c r="D98" s="3">
+        <v>1237</v>
+      </c>
+      <c r="E98" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" s="4">
+        <v>8.8477139999999999</v>
+      </c>
+      <c r="B99" s="4">
+        <v>-79.796204000000003</v>
+      </c>
+      <c r="C99" s="3">
+        <v>500</v>
+      </c>
+      <c r="D99" s="3">
+        <v>1238</v>
+      </c>
+      <c r="E99" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" s="4">
+        <v>8.0179720000000003</v>
+      </c>
+      <c r="B100" s="4">
+        <v>-81.327490999999995</v>
+      </c>
+      <c r="C100" s="3">
+        <v>500</v>
+      </c>
+      <c r="D100" s="3">
+        <v>1239</v>
+      </c>
+      <c r="E100" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" s="4">
+        <v>8.2394750000000005</v>
+      </c>
+      <c r="B101" s="4">
+        <v>-81.907392999999999</v>
+      </c>
+      <c r="C101" s="3">
+        <v>1000</v>
+      </c>
+      <c r="D101" s="3">
+        <v>1240</v>
+      </c>
+      <c r="E101" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" s="4">
+        <v>8.3660169999999994</v>
+      </c>
+      <c r="B102" s="4">
+        <v>-82.276599000000004</v>
+      </c>
+      <c r="C102" s="3">
+        <v>1000</v>
+      </c>
+      <c r="D102" s="3">
+        <v>1241</v>
+      </c>
+      <c r="E102" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" s="4">
+        <v>8.5368820000000003</v>
+      </c>
+      <c r="B103" s="4">
+        <v>-82.386922999999996</v>
+      </c>
+      <c r="C103" s="3">
+        <v>750</v>
+      </c>
+      <c r="D103" s="3">
+        <v>1242</v>
+      </c>
+      <c r="E103" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" s="4">
+        <v>8.6429329999999993</v>
+      </c>
+      <c r="B104" s="4">
+        <v>-80.511657</v>
+      </c>
+      <c r="C104" s="3">
+        <v>1000</v>
+      </c>
+      <c r="D104" s="3">
+        <v>1243</v>
+      </c>
+      <c r="E104" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" s="4">
+        <v>7.7252611729999998</v>
+      </c>
+      <c r="B105" s="4">
+        <v>-80.818248740000001</v>
+      </c>
+      <c r="C105" s="3">
+        <v>1500</v>
+      </c>
+      <c r="D105" s="3">
+        <v>1244</v>
+      </c>
+      <c r="E105" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" s="4">
+        <v>8.9090000000000007</v>
+      </c>
+      <c r="B106" s="4">
+        <v>-79.795000000000002</v>
+      </c>
+      <c r="C106" s="3">
+        <v>500</v>
+      </c>
+      <c r="D106" s="3">
+        <v>1245</v>
+      </c>
+      <c r="E106" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" s="4">
+        <v>8.9405999999999999</v>
+      </c>
+      <c r="B107" s="4">
+        <v>-79.656499999999994</v>
+      </c>
+      <c r="C107" s="3">
+        <v>500</v>
+      </c>
+      <c r="D107" s="3">
+        <v>1246</v>
+      </c>
+      <c r="E107" s="3">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix data input error. Add error handling
</commit_message>
<xml_diff>
--- a/locations.xlsx
+++ b/locations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\retro\repos\quest-rfi-new-sites\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4EE63BC-6B9E-4004-8638-2BD05ACADA4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AE37C98-81C7-4B02-9574-7380FBD4EAA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3210" yWindow="2970" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1267" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1266" uniqueCount="28">
   <si>
     <t>ID RFI</t>
   </si>
@@ -124,9 +124,6 @@
   </si>
   <si>
     <t>required_height</t>
-  </si>
-  <si>
-    <t>s</t>
   </si>
 </sst>
 </file>
@@ -533,8 +530,8 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>28</v>
+      <c r="A2" s="4">
+        <v>8.8932739999999999</v>
       </c>
       <c r="B2" s="4">
         <v>-79.620080999999999</v>

</xml_diff>